<commit_message>
Fix stock parsing for без-ЧЗ storage calc
Остаток во вкладке хранится текстом с неразрывным пробелом, из-за чего
8 товаров обнулялись. Парсер исправлен, итоги пересчитаны:
- на месяц: 189 455 руб (было 87 764)
- до ноября: 814 657 руб (было 377 387)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RrW5WcYKgjMut1vasTMe2Q
</commit_message>
<xml_diff>
--- a/outputs/Хранение_без_ЧЗ_месяц.xlsx
+++ b/outputs/Хранение_без_ЧЗ_месяц.xlsx
@@ -84,7 +84,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -94,6 +94,7 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -778,7 +779,7 @@
         </is>
       </c>
       <c r="C14" s="3" t="n">
-        <v>0</v>
+        <v>1108</v>
       </c>
       <c r="D14" s="4" t="n">
         <v>0.1545</v>
@@ -787,7 +788,7 @@
         <v>4.63</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>0</v>
+        <v>5135.58</v>
       </c>
     </row>
     <row r="15">
@@ -800,7 +801,7 @@
         </is>
       </c>
       <c r="C15" s="3" t="n">
-        <v>0</v>
+        <v>2515</v>
       </c>
       <c r="D15" s="4" t="n">
         <v>0.1355</v>
@@ -809,7 +810,7 @@
         <v>4.07</v>
       </c>
       <c r="F15" s="5" t="n">
-        <v>0</v>
+        <v>10223.48</v>
       </c>
     </row>
     <row r="16">
@@ -822,7 +823,7 @@
         </is>
       </c>
       <c r="C16" s="3" t="n">
-        <v>0</v>
+        <v>2757</v>
       </c>
       <c r="D16" s="4" t="n">
         <v>0.135</v>
@@ -831,7 +832,7 @@
         <v>4.05</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>0</v>
+        <v>11165.85</v>
       </c>
     </row>
     <row r="17">
@@ -910,7 +911,7 @@
         </is>
       </c>
       <c r="C20" s="3" t="n">
-        <v>0</v>
+        <v>1411</v>
       </c>
       <c r="D20" s="4" t="n">
         <v>0.1623</v>
@@ -919,7 +920,7 @@
         <v>4.87</v>
       </c>
       <c r="F20" s="5" t="n">
-        <v>0</v>
+        <v>6870.16</v>
       </c>
     </row>
     <row r="21">
@@ -1130,7 +1131,7 @@
         </is>
       </c>
       <c r="C30" s="3" t="n">
-        <v>0</v>
+        <v>3268</v>
       </c>
       <c r="D30" s="4" t="n">
         <v>0.3027</v>
@@ -1139,7 +1140,7 @@
         <v>9.08</v>
       </c>
       <c r="F30" s="5" t="n">
-        <v>0</v>
+        <v>29676.71</v>
       </c>
     </row>
     <row r="31">
@@ -1152,7 +1153,7 @@
         </is>
       </c>
       <c r="C31" s="3" t="n">
-        <v>0</v>
+        <v>4181</v>
       </c>
       <c r="D31" s="4" t="n">
         <v>0.2001</v>
@@ -1161,7 +1162,7 @@
         <v>6</v>
       </c>
       <c r="F31" s="5" t="n">
-        <v>0</v>
+        <v>25098.54</v>
       </c>
     </row>
     <row r="32">
@@ -1284,7 +1285,7 @@
         </is>
       </c>
       <c r="C37" s="3" t="n">
-        <v>0</v>
+        <v>1383</v>
       </c>
       <c r="D37" s="4" t="n">
         <v>0.1834</v>
@@ -1293,7 +1294,7 @@
         <v>5.5</v>
       </c>
       <c r="F37" s="5" t="n">
-        <v>0</v>
+        <v>7609.27</v>
       </c>
     </row>
     <row r="38">
@@ -1306,7 +1307,7 @@
         </is>
       </c>
       <c r="C38" s="3" t="n">
-        <v>0</v>
+        <v>1042</v>
       </c>
       <c r="D38" s="4" t="n">
         <v>0.1891</v>
@@ -1315,7 +1316,7 @@
         <v>5.67</v>
       </c>
       <c r="F38" s="5" t="n">
-        <v>0</v>
+        <v>5911.27</v>
       </c>
     </row>
     <row r="39">
@@ -1786,14 +1787,17 @@
           <t>ИТОГО</t>
         </is>
       </c>
-      <c r="F60" s="7" t="n">
-        <v>87764.37</v>
+      <c r="C60" s="7" t="n">
+        <v>33295</v>
+      </c>
+      <c r="F60" s="8" t="n">
+        <v>189455.23</v>
       </c>
     </row>
     <row r="62">
-      <c r="B62" s="8" t="inlineStr">
-        <is>
-          <t>Расчёт: хранение/мес за ед. = дневная ставка хранения за ед. (из файла платного хранения, сопоставлено по артикулу) × 30 дн. Хранение/мес всего = ставка/мес × остаток без ЧЗ. Значения посчитаны (без формул).</t>
+      <c r="B62" s="9" t="inlineStr">
+        <is>
+          <t>Хранение/мес = дневная ставка за ед. (файл хранения, по артикулу) × 30 дн × остаток без ЧЗ.</t>
         </is>
       </c>
     </row>

</xml_diff>